<commit_message>
[EN-135] mad correction and fix excel report error
</commit_message>
<xml_diff>
--- a/src/Envirotrax.App/Envirotrax.App.Server/Templates/Excel/Backflow/BackflowComplianceHistory.xlsx
+++ b/src/Envirotrax.App/Envirotrax.App.Server/Templates/Excel/Backflow/BackflowComplianceHistory.xlsx
@@ -984,29 +984,7 @@
       </border>
     </dxf>
   </dxfs>
-  <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
-    </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
-    </tableStyle>
-  </tableStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>

</xml_diff>